<commit_message>
Video_613: figuras regeneradas con el codigo nuevo (NO REPORTABLE en el titulo), mismos numeros
</commit_message>
<xml_diff>
--- a/data/processed_data/Video_613/contracciones.xlsx
+++ b/data/processed_data/Video_613/contracciones.xlsx
@@ -1176,8 +1176,8 @@
        'espontaneos', 'espontaneos', 'espontaneos', 'espontaneos'],
       dtype=object), 'tren_por_evento': array([0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0,
        0, 0]), 'estimulados': array([], dtype=int64), 'estimulados_dudosos': array([], dtype=int64), 'espontaneos': array([ 0,  1,  2,  3,  4,  5,  6,  7,  8,  9, 10, 11, 12, 13, 14, 15, 16,
-       17, 18, 19, 20, 21, 22, 23]), 'hay_estimulacion': False, 'n_trenes_estimulados': 0, 'tren_principal': 1, 'veredicto': 'no se encontro un tren periodico que se distinga del azar', 'z': 3.864, 'p_valor': 0.8971028971028971, 'periodo_grilla_s': 1.0633, 'periodo_s': 1.06694, 'periodo_err_s': 0.0061, 'frecuencia_Hz': 0.93726, 'frecuencia_err_Hz': 0.005357, 'jitter_s': 0.02196, 'tolerancia_s': 0.0667, 'n_estimulados': 4, 'n_ranuras': 6, 'tasa_captura_pct': 66.7, 'tren_inicio_s': 66.362, 'tren_fin_s': 71.706, 'motivo': 'no se encontro un tren periodico que se distinga del azar (mejor intento: T=1.067 s, z=3.86, p=0.897)', 'resumen_grupos':          grupo   n  t_inicio_s  ...  CV_intervalo_pct  amplitud_mediana_px  amplitud_IQR_px
-0  espontaneos  24        0.33  ...             283.5               0.3199           0.1223
+       17, 18, 19, 20, 21, 22, 23]), 'hay_estimulacion': False, 'n_trenes_estimulados': 0, 'tren_principal': 1, 'veredicto': 'no se encontro un tren periodico que se distinga del azar', 'z': 3.864, 'p_valor': 0.8971028971028971, 'periodo_grilla_s': 1.0633, 'periodo_s': 1.06694, 'periodo_err_s': 0.0061, 'frecuencia_Hz': 0.93726, 'frecuencia_err_Hz': 0.005357, 'jitter_s': 0.02196, 'tolerancia_s': 0.0667, 'n_estimulados': 4, 'n_ranuras': 6, 'tasa_captura_pct': 66.7, 'tren_inicio_s': 66.362, 'tren_fin_s': 71.706, 'motivo': 'no se encontro un tren periodico que se distinga del azar (mejor intento: T=1.067 s, z=3.86, p=0.897)', 'resumen_grupos':          grupo   n  ...  amplitud_mediana_px  amplitud_IQR_px
+0  espontaneos  24  ...               0.3199           0.1223
 [1 rows x 10 columns], 'espontaneas_instantanea':     tiempo_s  intervalo_s  frecuencia_Hz
 0      0.844       1.0270         0.9737
 1      1.689       0.6626         1.5091

</xml_diff>